<commit_message>
Add transform_size and use it in Try.py
Introduce code/pands.py with transform_size() to map detected pixels to real fish dimensions using Size_ikan.xlsx. Integrate the function in code/Try.py (import added) and apply species-specific transformations (nila/lele/mas) to compute transformed panjang/lebar (Pt,Lt), update perimeter and output prints to use the transformed values. Also include updated Size_ikan.xlsx, many rotated/boxed output images, and regenerated __pycache__ files.
</commit_message>
<xml_diff>
--- a/Size_ikan.xlsx
+++ b/Size_ikan.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="21">
   <si>
     <t>no</t>
   </si>
@@ -39,7 +39,46 @@
     <t>rata-rata berat/keliling ikan</t>
   </si>
   <si>
-    <t>No</t>
+    <t>nama_file</t>
+  </si>
+  <si>
+    <t>Ikan_Nila_induk_1</t>
+  </si>
+  <si>
+    <t>Ikan_Nila_induk_2</t>
+  </si>
+  <si>
+    <t>Ikan_Nila_induk_3</t>
+  </si>
+  <si>
+    <t>Ikan_Nila_kdua_4</t>
+  </si>
+  <si>
+    <t>Ikan_Nila_kdua_5</t>
+  </si>
+  <si>
+    <t>Ikan_Nila_kdua_6</t>
+  </si>
+  <si>
+    <t>Ikan_Nila_kdua_7</t>
+  </si>
+  <si>
+    <t>Ikan_Nila_kdua_8</t>
+  </si>
+  <si>
+    <t>Ikan_Nila_Kbawah_9</t>
+  </si>
+  <si>
+    <t>Ikan_Nila_Kbawah_10</t>
+  </si>
+  <si>
+    <t>Ikan_Nila_Kbawah_11</t>
+  </si>
+  <si>
+    <t>Ikan_Nila_Kbawah_12</t>
+  </si>
+  <si>
+    <t>Ikan_Nila_Kbawah_13</t>
   </si>
 </sst>
 </file>
@@ -63,7 +102,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -206,7 +245,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="32">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -214,107 +253,92 @@
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="4" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="5" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="6" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="5" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="7" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="8" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="9" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="8" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="10" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="4" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="5" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="6" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="5" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="7" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="8" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="9" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="8" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="10" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="10" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="5" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="5" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="6" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="8" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="9" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="10" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="5" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="6" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="8" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="9" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="10" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="10" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="10" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="10" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="10" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="10" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="5" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="10" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="10" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="10" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="10" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -364,7 +388,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:F14" displayName="Table1" name="Table1" id="3" totalsRowShown="0">
   <autoFilter ref="A1:F14"/>
   <tableColumns count="6">
-    <tableColumn name="No" id="1"/>
+    <tableColumn name="nama_file" id="1"/>
     <tableColumn name="panjang" id="2"/>
     <tableColumn name="lebar" id="3"/>
     <tableColumn name="berat" id="4"/>
@@ -666,313 +690,313 @@
   <dimension ref="A1:F16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="31" width="22.862142857142857" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="22.5">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="30" t="s">
+      <c r="B1" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="31" t="s">
+      <c r="C1" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="30" t="s">
+      <c r="D1" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="32" t="s">
+      <c r="E1" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="33" t="s">
+      <c r="F1" s="27" t="s">
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="22.5">
-      <c r="A2" s="34">
-        <v>1</v>
-      </c>
-      <c r="B2" s="34">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
+      <c r="A2" s="28" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="29">
         <v>33</v>
       </c>
-      <c r="C2" s="34">
+      <c r="C2" s="29">
         <v>14</v>
       </c>
-      <c r="D2" s="34">
+      <c r="D2" s="29">
         <v>670</v>
       </c>
-      <c r="E2" s="35">
+      <c r="E2" s="16">
         <f>2*(Table1[[#This Row], [panjang]]+Table1[[#This Row], [lebar]])</f>
       </c>
-      <c r="F2" s="36">
+      <c r="F2" s="15">
         <f>Table1[[#This Row], [berat]]/Table1[[#This Row], [keliling]]</f>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="22.5">
-      <c r="A3" s="34">
-        <v>2</v>
-      </c>
-      <c r="B3" s="34">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
+      <c r="A3" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="29">
         <v>31</v>
       </c>
-      <c r="C3" s="34">
+      <c r="C3" s="29">
         <v>12</v>
       </c>
-      <c r="D3" s="34">
+      <c r="D3" s="29">
         <v>450</v>
       </c>
-      <c r="E3" s="35">
+      <c r="E3" s="16">
         <f>2*(Table1[[#This Row], [panjang]]+Table1[[#This Row], [lebar]])</f>
       </c>
-      <c r="F3" s="36">
+      <c r="F3" s="15">
         <f>Table1[[#This Row], [berat]]/Table1[[#This Row], [keliling]]</f>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="22.5">
-      <c r="A4" s="34">
-        <v>3</v>
-      </c>
-      <c r="B4" s="34">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
+      <c r="A4" s="28" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="29">
         <v>28</v>
       </c>
-      <c r="C4" s="34">
+      <c r="C4" s="29">
         <v>11</v>
       </c>
-      <c r="D4" s="34">
+      <c r="D4" s="29">
         <v>370</v>
       </c>
-      <c r="E4" s="35">
+      <c r="E4" s="16">
         <f>2*(Table1[[#This Row], [panjang]]+Table1[[#This Row], [lebar]])</f>
       </c>
-      <c r="F4" s="36">
+      <c r="F4" s="15">
         <f>Table1[[#This Row], [berat]]/Table1[[#This Row], [keliling]]</f>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="22.5">
-      <c r="A5" s="34">
-        <v>4</v>
-      </c>
-      <c r="B5" s="34">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
+      <c r="A5" s="28" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="29">
         <v>19</v>
       </c>
-      <c r="C5" s="34">
+      <c r="C5" s="29">
         <v>6</v>
       </c>
-      <c r="D5" s="34">
+      <c r="D5" s="29">
         <v>135</v>
       </c>
-      <c r="E5" s="35">
+      <c r="E5" s="16">
         <f>2*(Table1[[#This Row], [panjang]]+Table1[[#This Row], [lebar]])</f>
       </c>
-      <c r="F5" s="36">
+      <c r="F5" s="15">
         <f>Table1[[#This Row], [berat]]/Table1[[#This Row], [keliling]]</f>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="22.5">
-      <c r="A6" s="34">
-        <v>5</v>
-      </c>
-      <c r="B6" s="34">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
+      <c r="A6" s="28" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="29">
         <v>25</v>
       </c>
-      <c r="C6" s="34">
+      <c r="C6" s="29">
         <v>9</v>
       </c>
-      <c r="D6" s="34">
+      <c r="D6" s="29">
         <v>260</v>
       </c>
-      <c r="E6" s="35">
+      <c r="E6" s="16">
         <f>2*(Table1[[#This Row], [panjang]]+Table1[[#This Row], [lebar]])</f>
       </c>
-      <c r="F6" s="36">
+      <c r="F6" s="15">
         <f>Table1[[#This Row], [berat]]/Table1[[#This Row], [keliling]]</f>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="22.5">
-      <c r="A7" s="34">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
+      <c r="A7" s="28" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="29">
+        <v>23</v>
+      </c>
+      <c r="C7" s="29">
+        <v>8</v>
+      </c>
+      <c r="D7" s="29">
+        <v>225</v>
+      </c>
+      <c r="E7" s="16">
+        <f>2*(Table1[[#This Row], [panjang]]+Table1[[#This Row], [lebar]])</f>
+      </c>
+      <c r="F7" s="15">
+        <f>Table1[[#This Row], [berat]]/Table1[[#This Row], [keliling]]</f>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
+      <c r="A8" s="28" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="29">
+        <v>24</v>
+      </c>
+      <c r="C8" s="29">
+        <v>8</v>
+      </c>
+      <c r="D8" s="29">
+        <v>220</v>
+      </c>
+      <c r="E8" s="16">
+        <f>2*(Table1[[#This Row], [panjang]]+Table1[[#This Row], [lebar]])</f>
+      </c>
+      <c r="F8" s="15">
+        <f>Table1[[#This Row], [berat]]/Table1[[#This Row], [keliling]]</f>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
+      <c r="A9" s="28" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="29">
+        <v>24</v>
+      </c>
+      <c r="C9" s="29">
+        <v>8</v>
+      </c>
+      <c r="D9" s="29">
+        <v>200</v>
+      </c>
+      <c r="E9" s="16">
+        <f>2*(Table1[[#This Row], [panjang]]+Table1[[#This Row], [lebar]])</f>
+      </c>
+      <c r="F9" s="15">
+        <f>Table1[[#This Row], [berat]]/Table1[[#This Row], [keliling]]</f>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
+      <c r="A10" s="28" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="29">
+        <v>24</v>
+      </c>
+      <c r="C10" s="29">
+        <v>7</v>
+      </c>
+      <c r="D10" s="29">
+        <v>180</v>
+      </c>
+      <c r="E10" s="16">
+        <f>2*(Table1[[#This Row], [panjang]]+Table1[[#This Row], [lebar]])</f>
+      </c>
+      <c r="F10" s="15">
+        <f>Table1[[#This Row], [berat]]/Table1[[#This Row], [keliling]]</f>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
+      <c r="A11" s="28" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="29">
+        <v>22</v>
+      </c>
+      <c r="C11" s="29">
+        <v>8</v>
+      </c>
+      <c r="D11" s="29">
+        <v>180</v>
+      </c>
+      <c r="E11" s="16">
+        <f>2*(Table1[[#This Row], [panjang]]+Table1[[#This Row], [lebar]])</f>
+      </c>
+      <c r="F11" s="16">
+        <f>Table1[[#This Row], [berat]]/Table1[[#This Row], [keliling]]</f>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
+      <c r="A12" s="28" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="29">
+        <v>20</v>
+      </c>
+      <c r="C12" s="29">
+        <v>7</v>
+      </c>
+      <c r="D12" s="29">
+        <v>160</v>
+      </c>
+      <c r="E12" s="16">
+        <f>2*(Table1[[#This Row], [panjang]]+Table1[[#This Row], [lebar]])</f>
+      </c>
+      <c r="F12" s="15">
+        <f>Table1[[#This Row], [berat]]/Table1[[#This Row], [keliling]]</f>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
+      <c r="A13" s="28" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" s="29">
+        <v>19</v>
+      </c>
+      <c r="C13" s="29">
+        <v>7</v>
+      </c>
+      <c r="D13" s="29">
+        <v>120</v>
+      </c>
+      <c r="E13" s="16">
+        <f>2*(Table1[[#This Row], [panjang]]+Table1[[#This Row], [lebar]])</f>
+      </c>
+      <c r="F13" s="15">
+        <f>Table1[[#This Row], [berat]]/Table1[[#This Row], [keliling]]</f>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
+      <c r="A14" s="28" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="29">
+        <v>20</v>
+      </c>
+      <c r="C14" s="29">
         <v>6</v>
       </c>
-      <c r="B7" s="34">
-        <v>23</v>
-      </c>
-      <c r="C7" s="34">
-        <v>8</v>
-      </c>
-      <c r="D7" s="34">
-        <v>225</v>
-      </c>
-      <c r="E7" s="35">
+      <c r="D14" s="29">
+        <v>140</v>
+      </c>
+      <c r="E14" s="16">
         <f>2*(Table1[[#This Row], [panjang]]+Table1[[#This Row], [lebar]])</f>
       </c>
-      <c r="F7" s="36">
+      <c r="F14" s="15">
         <f>Table1[[#This Row], [berat]]/Table1[[#This Row], [keliling]]</f>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="22.5">
-      <c r="A8" s="34">
-        <v>7</v>
-      </c>
-      <c r="B8" s="34">
-        <v>24</v>
-      </c>
-      <c r="C8" s="34">
-        <v>8</v>
-      </c>
-      <c r="D8" s="34">
-        <v>220</v>
-      </c>
-      <c r="E8" s="35">
-        <f>2*(Table1[[#This Row], [panjang]]+Table1[[#This Row], [lebar]])</f>
-      </c>
-      <c r="F8" s="36">
-        <f>Table1[[#This Row], [berat]]/Table1[[#This Row], [keliling]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="22.5">
-      <c r="A9" s="34">
-        <v>8</v>
-      </c>
-      <c r="B9" s="34">
-        <v>24</v>
-      </c>
-      <c r="C9" s="34">
-        <v>8</v>
-      </c>
-      <c r="D9" s="34">
-        <v>200</v>
-      </c>
-      <c r="E9" s="35">
-        <f>2*(Table1[[#This Row], [panjang]]+Table1[[#This Row], [lebar]])</f>
-      </c>
-      <c r="F9" s="36">
-        <f>Table1[[#This Row], [berat]]/Table1[[#This Row], [keliling]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="22.5">
-      <c r="A10" s="34">
-        <v>9</v>
-      </c>
-      <c r="B10" s="34">
-        <v>24</v>
-      </c>
-      <c r="C10" s="34">
-        <v>7</v>
-      </c>
-      <c r="D10" s="34">
-        <v>180</v>
-      </c>
-      <c r="E10" s="35">
-        <f>2*(Table1[[#This Row], [panjang]]+Table1[[#This Row], [lebar]])</f>
-      </c>
-      <c r="F10" s="36">
-        <f>Table1[[#This Row], [berat]]/Table1[[#This Row], [keliling]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="22.5">
-      <c r="A11" s="34">
-        <v>10</v>
-      </c>
-      <c r="B11" s="34">
-        <v>22</v>
-      </c>
-      <c r="C11" s="34">
-        <v>8</v>
-      </c>
-      <c r="D11" s="34">
-        <v>180</v>
-      </c>
-      <c r="E11" s="35">
-        <f>2*(Table1[[#This Row], [panjang]]+Table1[[#This Row], [lebar]])</f>
-      </c>
-      <c r="F11" s="35">
-        <f>Table1[[#This Row], [berat]]/Table1[[#This Row], [keliling]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="22.5">
-      <c r="A12" s="34">
-        <v>11</v>
-      </c>
-      <c r="B12" s="34">
-        <v>20</v>
-      </c>
-      <c r="C12" s="34">
-        <v>7</v>
-      </c>
-      <c r="D12" s="34">
-        <v>160</v>
-      </c>
-      <c r="E12" s="35">
-        <f>2*(Table1[[#This Row], [panjang]]+Table1[[#This Row], [lebar]])</f>
-      </c>
-      <c r="F12" s="36">
-        <f>Table1[[#This Row], [berat]]/Table1[[#This Row], [keliling]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="22.5">
-      <c r="A13" s="34">
-        <v>12</v>
-      </c>
-      <c r="B13" s="34">
-        <v>19</v>
-      </c>
-      <c r="C13" s="34">
-        <v>7</v>
-      </c>
-      <c r="D13" s="34">
-        <v>120</v>
-      </c>
-      <c r="E13" s="35">
-        <f>2*(Table1[[#This Row], [panjang]]+Table1[[#This Row], [lebar]])</f>
-      </c>
-      <c r="F13" s="36">
-        <f>Table1[[#This Row], [berat]]/Table1[[#This Row], [keliling]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="22.5">
-      <c r="A14" s="34">
-        <v>13</v>
-      </c>
-      <c r="B14" s="34">
-        <v>20</v>
-      </c>
-      <c r="C14" s="34">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
+      <c r="A15" s="14"/>
+      <c r="B15" s="14"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="15"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="20.25">
+      <c r="A16" s="30" t="s">
         <v>6</v>
       </c>
-      <c r="D14" s="34">
-        <v>140</v>
-      </c>
-      <c r="E14" s="35">
-        <f>2*(Table1[[#This Row], [panjang]]+Table1[[#This Row], [lebar]])</f>
-      </c>
-      <c r="F14" s="36">
-        <f>Table1[[#This Row], [berat]]/Table1[[#This Row], [keliling]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
-      <c r="A15" s="15"/>
-      <c r="B15" s="15"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="17"/>
-      <c r="F15" s="18"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="15.75">
-      <c r="A16" s="19" t="s">
-        <v>6</v>
-      </c>
-      <c r="B16" s="19"/>
-      <c r="C16" s="10">
+      <c r="B16" s="17"/>
+      <c r="C16" s="9">
         <f>AVERAGE(Table1[berat/keliling])</f>
       </c>
-      <c r="D16" s="17"/>
-      <c r="E16" s="17"/>
-      <c r="F16" s="18"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -993,12 +1017,12 @@
   <dimension ref="A1:F17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="23" width="19.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="20" width="19.14785714285714" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="22.5">
@@ -1008,306 +1032,306 @@
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="24" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="25" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="22.5">
-      <c r="A2" s="6">
+      <c r="A2" s="5">
         <v>1</v>
       </c>
-      <c r="B2" s="7">
+      <c r="B2" s="6">
         <v>52</v>
       </c>
-      <c r="C2" s="7">
+      <c r="C2" s="6">
         <v>8</v>
       </c>
-      <c r="D2" s="7">
+      <c r="D2" s="6">
         <v>830</v>
       </c>
-      <c r="E2" s="26">
+      <c r="E2" s="21">
         <f>2*(Table3[[#This Row], [panjang]]+Table3[[#This Row], [lebar]])</f>
       </c>
-      <c r="F2" s="27">
+      <c r="F2" s="22">
         <f>Table3[[#This Row], [berat]]/Table3[[#This Row], [keliling]]</f>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="22.5">
-      <c r="A3" s="6">
+      <c r="A3" s="5">
         <v>2</v>
       </c>
-      <c r="B3" s="7">
+      <c r="B3" s="6">
         <v>54</v>
       </c>
-      <c r="C3" s="7">
+      <c r="C3" s="6">
         <v>9</v>
       </c>
-      <c r="D3" s="7">
+      <c r="D3" s="6">
         <v>940</v>
       </c>
-      <c r="E3" s="26">
+      <c r="E3" s="21">
         <f>2*(Table3[[#This Row], [panjang]]+Table3[[#This Row], [lebar]])</f>
       </c>
-      <c r="F3" s="27">
+      <c r="F3" s="22">
         <f>Table3[[#This Row], [berat]]/Table3[[#This Row], [keliling]]</f>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="22.5">
-      <c r="A4" s="6">
+      <c r="A4" s="5">
         <v>3</v>
       </c>
-      <c r="B4" s="7">
+      <c r="B4" s="6">
         <v>53</v>
       </c>
-      <c r="C4" s="7">
+      <c r="C4" s="6">
         <v>8</v>
       </c>
-      <c r="D4" s="7">
+      <c r="D4" s="6">
         <v>880</v>
       </c>
-      <c r="E4" s="26">
+      <c r="E4" s="21">
         <f>2*(Table3[[#This Row], [panjang]]+Table3[[#This Row], [lebar]])</f>
       </c>
-      <c r="F4" s="27">
+      <c r="F4" s="22">
         <f>Table3[[#This Row], [berat]]/Table3[[#This Row], [keliling]]</f>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="22.5">
-      <c r="A5" s="6">
+      <c r="A5" s="5">
         <v>4</v>
       </c>
-      <c r="B5" s="7">
+      <c r="B5" s="6">
         <v>39</v>
       </c>
-      <c r="C5" s="7">
+      <c r="C5" s="6">
         <v>7</v>
       </c>
-      <c r="D5" s="7">
+      <c r="D5" s="6">
         <v>430</v>
       </c>
-      <c r="E5" s="26">
+      <c r="E5" s="21">
         <f>2*(Table3[[#This Row], [panjang]]+Table3[[#This Row], [lebar]])</f>
       </c>
-      <c r="F5" s="27">
+      <c r="F5" s="22">
         <f>Table3[[#This Row], [berat]]/Table3[[#This Row], [keliling]]</f>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="22.5">
-      <c r="A6" s="6">
+      <c r="A6" s="5">
         <v>5</v>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="6">
         <v>41</v>
       </c>
-      <c r="C6" s="7">
+      <c r="C6" s="6">
         <v>7</v>
       </c>
-      <c r="D6" s="7">
+      <c r="D6" s="6">
         <v>460</v>
       </c>
-      <c r="E6" s="26">
+      <c r="E6" s="21">
         <f>2*(Table3[[#This Row], [panjang]]+Table3[[#This Row], [lebar]])</f>
       </c>
-      <c r="F6" s="27">
+      <c r="F6" s="22">
         <f>Table3[[#This Row], [berat]]/Table3[[#This Row], [keliling]]</f>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="22.5">
-      <c r="A7" s="6">
+      <c r="A7" s="5">
         <v>6</v>
       </c>
-      <c r="B7" s="7">
+      <c r="B7" s="6">
         <v>35</v>
       </c>
-      <c r="C7" s="7">
+      <c r="C7" s="6">
         <v>6</v>
       </c>
-      <c r="D7" s="7">
+      <c r="D7" s="6">
         <v>350</v>
       </c>
-      <c r="E7" s="26">
+      <c r="E7" s="21">
         <f>2*(Table3[[#This Row], [panjang]]+Table3[[#This Row], [lebar]])</f>
       </c>
-      <c r="F7" s="27">
+      <c r="F7" s="22">
         <f>Table3[[#This Row], [berat]]/Table3[[#This Row], [keliling]]</f>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="22.5">
-      <c r="A8" s="6">
+      <c r="A8" s="5">
         <v>7</v>
       </c>
-      <c r="B8" s="7">
+      <c r="B8" s="6">
         <v>35</v>
       </c>
-      <c r="C8" s="7">
+      <c r="C8" s="6">
         <v>6</v>
       </c>
-      <c r="D8" s="7">
+      <c r="D8" s="6">
         <v>320</v>
       </c>
-      <c r="E8" s="26">
+      <c r="E8" s="21">
         <f>2*(Table3[[#This Row], [panjang]]+Table3[[#This Row], [lebar]])</f>
       </c>
-      <c r="F8" s="27">
+      <c r="F8" s="22">
         <f>Table3[[#This Row], [berat]]/Table3[[#This Row], [keliling]]</f>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="22.5">
-      <c r="A9" s="6">
+      <c r="A9" s="5">
         <v>8</v>
       </c>
-      <c r="B9" s="7">
+      <c r="B9" s="6">
         <v>28</v>
       </c>
-      <c r="C9" s="7">
+      <c r="C9" s="6">
         <v>6</v>
       </c>
-      <c r="D9" s="7">
+      <c r="D9" s="6">
         <v>140</v>
       </c>
-      <c r="E9" s="26">
+      <c r="E9" s="21">
         <f>2*(Table3[[#This Row], [panjang]]+Table3[[#This Row], [lebar]])</f>
       </c>
-      <c r="F9" s="27">
+      <c r="F9" s="22">
         <f>Table3[[#This Row], [berat]]/Table3[[#This Row], [keliling]]</f>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="22.5">
-      <c r="A10" s="6">
+      <c r="A10" s="5">
         <v>9</v>
       </c>
-      <c r="B10" s="7">
+      <c r="B10" s="6">
         <v>27</v>
       </c>
-      <c r="C10" s="7">
+      <c r="C10" s="6">
         <v>6</v>
       </c>
-      <c r="D10" s="7">
+      <c r="D10" s="6">
         <v>160</v>
       </c>
-      <c r="E10" s="26">
+      <c r="E10" s="21">
         <f>2*(Table3[[#This Row], [panjang]]+Table3[[#This Row], [lebar]])</f>
       </c>
-      <c r="F10" s="27">
+      <c r="F10" s="22">
         <f>Table3[[#This Row], [berat]]/Table3[[#This Row], [keliling]]</f>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="22.5">
-      <c r="A11" s="6">
+      <c r="A11" s="5">
         <v>10</v>
       </c>
-      <c r="B11" s="7">
+      <c r="B11" s="6">
         <v>27</v>
       </c>
-      <c r="C11" s="7">
+      <c r="C11" s="6">
         <v>5</v>
       </c>
-      <c r="D11" s="7">
+      <c r="D11" s="6">
         <v>100</v>
       </c>
-      <c r="E11" s="26">
+      <c r="E11" s="21">
         <f>2*(Table3[[#This Row], [panjang]]+Table3[[#This Row], [lebar]])</f>
       </c>
-      <c r="F11" s="27">
+      <c r="F11" s="22">
         <f>Table3[[#This Row], [berat]]/Table3[[#This Row], [keliling]]</f>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="22.5">
-      <c r="A12" s="6">
+      <c r="A12" s="5">
         <v>11</v>
       </c>
-      <c r="B12" s="7">
+      <c r="B12" s="6">
         <v>25</v>
       </c>
-      <c r="C12" s="7">
+      <c r="C12" s="6">
         <v>6</v>
       </c>
-      <c r="D12" s="7">
+      <c r="D12" s="6">
         <v>120</v>
       </c>
-      <c r="E12" s="26">
+      <c r="E12" s="21">
         <f>2*(Table3[[#This Row], [panjang]]+Table3[[#This Row], [lebar]])</f>
       </c>
-      <c r="F12" s="27">
+      <c r="F12" s="22">
         <f>Table3[[#This Row], [berat]]/Table3[[#This Row], [keliling]]</f>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="22.5">
-      <c r="A13" s="6">
+      <c r="A13" s="5">
         <v>12</v>
       </c>
-      <c r="B13" s="7">
+      <c r="B13" s="6">
         <v>20</v>
       </c>
-      <c r="C13" s="7">
+      <c r="C13" s="6">
         <v>6</v>
       </c>
-      <c r="D13" s="7">
+      <c r="D13" s="6">
         <v>220</v>
       </c>
-      <c r="E13" s="26">
+      <c r="E13" s="21">
         <f>2*(Table3[[#This Row], [panjang]]+Table3[[#This Row], [lebar]])</f>
       </c>
-      <c r="F13" s="27">
+      <c r="F13" s="22">
         <f>Table3[[#This Row], [berat]]/Table3[[#This Row], [keliling]]</f>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="22.5">
-      <c r="A14" s="11">
+      <c r="A14" s="10">
         <v>13</v>
       </c>
-      <c r="B14" s="12">
+      <c r="B14" s="11">
         <v>28</v>
       </c>
-      <c r="C14" s="12">
+      <c r="C14" s="11">
         <v>5</v>
       </c>
-      <c r="D14" s="12">
+      <c r="D14" s="11">
         <v>170</v>
       </c>
-      <c r="E14" s="28">
+      <c r="E14" s="23">
         <f>2*(Table3[[#This Row], [panjang]]+Table3[[#This Row], [lebar]])</f>
       </c>
-      <c r="F14" s="29">
+      <c r="F14" s="24">
         <f>Table3[[#This Row], [berat]]/Table3[[#This Row], [keliling]]</f>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
-      <c r="A15" s="15"/>
-      <c r="B15" s="15"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="17"/>
-      <c r="F15" s="18"/>
+      <c r="A15" s="14"/>
+      <c r="B15" s="14"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="15"/>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
-      <c r="A16" s="15"/>
-      <c r="B16" s="15"/>
-      <c r="C16" s="16"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="17"/>
-      <c r="F16" s="18"/>
+      <c r="A16" s="14"/>
+      <c r="B16" s="14"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="15"/>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="15.75">
-      <c r="A17" s="19" t="s">
+      <c r="A17" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="B17" s="19"/>
-      <c r="C17" s="10">
+      <c r="B17" s="17"/>
+      <c r="C17" s="9">
         <f>AVERAGE(Table3[berat/keliling])</f>
       </c>
-      <c r="D17" s="17"/>
-      <c r="E17" s="17"/>
-      <c r="F17" s="18"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="16"/>
+      <c r="F17" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1328,12 +1352,12 @@
   <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="21" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="22" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="23" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="18" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="19" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="20" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="22.5">
@@ -1343,158 +1367,158 @@
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="6">
+      <c r="A2" s="5">
         <v>1</v>
       </c>
-      <c r="B2" s="7">
+      <c r="B2" s="6">
         <v>34</v>
       </c>
-      <c r="C2" s="7">
+      <c r="C2" s="6">
         <v>14</v>
       </c>
-      <c r="D2" s="7">
+      <c r="D2" s="6">
         <v>740</v>
       </c>
-      <c r="E2" s="8">
+      <c r="E2" s="7">
         <f>2*(Table2[[#This Row], [panjang]]+Table2[[#This Row], [lebar]])</f>
       </c>
-      <c r="F2" s="9">
+      <c r="F2" s="8">
         <f>Table2[[#This Row], [berat]]/Table2[[#This Row], [keliling]]</f>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="6">
+      <c r="A3" s="5">
         <v>2</v>
       </c>
-      <c r="B3" s="7">
+      <c r="B3" s="6">
         <v>29</v>
       </c>
-      <c r="C3" s="7">
+      <c r="C3" s="6">
         <v>12</v>
       </c>
-      <c r="D3" s="7">
+      <c r="D3" s="6">
         <v>500</v>
       </c>
-      <c r="E3" s="8">
+      <c r="E3" s="7">
         <f>2*(Table2[[#This Row], [panjang]]+Table2[[#This Row], [lebar]])</f>
       </c>
-      <c r="F3" s="10">
+      <c r="F3" s="9">
         <f>Table2[[#This Row], [berat]]/Table2[[#This Row], [keliling]]</f>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="6">
+      <c r="A4" s="5">
         <v>3</v>
       </c>
-      <c r="B4" s="7">
+      <c r="B4" s="6">
         <v>37</v>
       </c>
-      <c r="C4" s="7">
+      <c r="C4" s="6">
         <v>12</v>
       </c>
-      <c r="D4" s="7">
+      <c r="D4" s="6">
         <v>764</v>
       </c>
-      <c r="E4" s="8">
+      <c r="E4" s="7">
         <f>2*(Table2[[#This Row], [panjang]]+Table2[[#This Row], [lebar]])</f>
       </c>
-      <c r="F4" s="10">
+      <c r="F4" s="9">
         <f>Table2[[#This Row], [berat]]/Table2[[#This Row], [keliling]]</f>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="6">
+      <c r="A5" s="5">
         <v>4</v>
       </c>
-      <c r="B5" s="7">
+      <c r="B5" s="6">
         <v>31</v>
       </c>
-      <c r="C5" s="7">
+      <c r="C5" s="6">
         <v>10</v>
       </c>
-      <c r="D5" s="7">
+      <c r="D5" s="6">
         <v>464</v>
       </c>
-      <c r="E5" s="8">
+      <c r="E5" s="7">
         <f>2*(Table2[[#This Row], [panjang]]+Table2[[#This Row], [lebar]])</f>
       </c>
-      <c r="F5" s="10">
+      <c r="F5" s="9">
         <f>Table2[[#This Row], [berat]]/Table2[[#This Row], [keliling]]</f>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
-      <c r="A6" s="6">
+      <c r="A6" s="5">
         <v>5</v>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="6">
         <v>24</v>
       </c>
-      <c r="C6" s="7">
+      <c r="C6" s="6">
         <v>7</v>
       </c>
-      <c r="D6" s="7">
+      <c r="D6" s="6">
         <v>230</v>
       </c>
-      <c r="E6" s="8">
+      <c r="E6" s="7">
         <f>2*(Table2[[#This Row], [panjang]]+Table2[[#This Row], [lebar]])</f>
       </c>
-      <c r="F6" s="10">
+      <c r="F6" s="9">
         <f>Table2[[#This Row], [berat]]/Table2[[#This Row], [keliling]]</f>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
-      <c r="A7" s="11">
+      <c r="A7" s="10">
         <v>6</v>
       </c>
-      <c r="B7" s="12">
+      <c r="B7" s="11">
         <v>26</v>
       </c>
-      <c r="C7" s="12">
+      <c r="C7" s="11">
         <v>8</v>
       </c>
-      <c r="D7" s="12">
+      <c r="D7" s="11">
         <v>312</v>
       </c>
-      <c r="E7" s="13">
+      <c r="E7" s="12">
         <f>2*(Table2[[#This Row], [panjang]]+Table2[[#This Row], [lebar]])</f>
       </c>
-      <c r="F7" s="14">
+      <c r="F7" s="13">
         <f>Table2[[#This Row], [berat]]/Table2[[#This Row], [keliling]]</f>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
-      <c r="A8" s="15"/>
-      <c r="B8" s="15"/>
-      <c r="C8" s="16"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="17"/>
-      <c r="F8" s="18"/>
+      <c r="A8" s="14"/>
+      <c r="B8" s="14"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="15"/>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="19"/>
-      <c r="C9" s="10">
+      <c r="B9" s="17"/>
+      <c r="C9" s="9">
         <f>AVERAGE(Table2[berat/keliling])</f>
       </c>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="18"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>